<commit_message>
Write the K ranges of the Bank and Corporate Rating test workbooks in digits (EPBDS-9967) and start the WS container with IF_ABSENT instead of the removed true
</commit_message>
<xml_diff>
--- a/src/test/resources/ruleservice_repo/TestWebservicesDeployUI/SimpleProject/SimpleProject/Bank Rating.xlsx
+++ b/src/test/resources/ruleservice_repo/TestWebservicesDeployUI/SimpleProject/SimpleProject/Bank Rating.xlsx
@@ -2320,25 +2320,25 @@
          Components of the qualitative analysis are monitoring of bank-counterparty’s ratings assigned by international rating agencies, the existence and nature of the bank's credit history, current level of relationships with the bank, its shareholders and management, the business reputational analysis of the bank, monitoring of relations with a financial supervisory authority.</t>
   </si>
   <si>
-    <t>&lt; 8K</t>
-  </si>
-  <si>
-    <t>[8K .. 100K)</t>
-  </si>
-  <si>
-    <t>&gt;= 100K</t>
-  </si>
-  <si>
-    <t>&lt; 1K</t>
-  </si>
-  <si>
-    <t>[1K .. 10K)</t>
-  </si>
-  <si>
-    <t>&gt;= 10K</t>
-  </si>
-  <si>
-    <t>&lt; 2K</t>
+    <t>&lt; 8000</t>
+  </si>
+  <si>
+    <t>[8000 .. 100000)</t>
+  </si>
+  <si>
+    <t>&gt;= 100000</t>
+  </si>
+  <si>
+    <t>&lt; 1000</t>
+  </si>
+  <si>
+    <t>[1000 .. 10000)</t>
+  </si>
+  <si>
+    <t>&gt;= 10000</t>
+  </si>
+  <si>
+    <t>&lt; 2000</t>
   </si>
   <si>
     <t>&gt;= 600</t>
@@ -2350,19 +2350,19 @@
     <t>&lt; 200</t>
   </si>
   <si>
-    <t>&gt; 1K</t>
-  </si>
-  <si>
-    <t>[200 .. 1K]</t>
+    <t>&gt; 1000</t>
+  </si>
+  <si>
+    <t>[200 .. 1000]</t>
   </si>
   <si>
     <t>DE</t>
   </si>
   <si>
-    <t>[2K .. 30K)</t>
-  </si>
-  <si>
-    <t>&gt;= 30K</t>
+    <t>[2000 .. 30000)</t>
+  </si>
+  <si>
+    <t>&gt;= 30000</t>
   </si>
   <si>
     <t>BE</t>

</xml_diff>